<commit_message>
Deploying to gh-pages from @ pedalboard/pedalboard-display@557fe1e7ba489c80f5472a749895be0239d2892c 🚀
</commit_message>
<xml_diff>
--- a/latest/BoM/Costs/pedalboard-display-bom.xlsx
+++ b/latest/BoM/Costs/pedalboard-display-bom.xlsx
@@ -484,7 +484,7 @@
     <t>KiCad Version:</t>
   </si>
   <si>
-    <t>9.0.7+1</t>
+    <t>10.0.1-10.0.1~ubuntu25.10.1</t>
   </si>
   <si>
     <t>Component Groups:</t>
@@ -559,10 +559,10 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2026-04-21 20:44:23</t>
-  </si>
-  <si>
-    <t>KiCost® v1.1.20 + KiBot v1.8.5</t>
+    <t>2026-04-22 17:54:39</t>
+  </si>
+  <si>
+    <t>KiCost® v1.1.20 + KiBot v1.8.6</t>
   </si>
   <si>
     <t>Resistor</t>
@@ -1780,7 +1780,7 @@
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
     <col min="2" max="2" width="21.7109375" customWidth="1"/>
     <col min="3" max="3" width="19.7109375" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="4" max="4" width="27.7109375" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="51.7109375" customWidth="1"/>
     <col min="7" max="7" width="26.7109375" customWidth="1"/>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ pedalboard/pedalboard-display@433e9090f67a40721300e903c0206a3a29c8822a 🚀
</commit_message>
<xml_diff>
--- a/latest/BoM/Costs/pedalboard-display-bom.xlsx
+++ b/latest/BoM/Costs/pedalboard-display-bom.xlsx
@@ -559,10 +559,10 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2026-05-12 07:16:41</t>
-  </si>
-  <si>
-    <t>KiCost® v1.1.20 + KiBot v1.8.6</t>
+    <t>2026-05-13 11:35:33</t>
+  </si>
+  <si>
+    <t>KiCost® v1.1.20 + KiBot v1.9.0</t>
   </si>
   <si>
     <t>Resistor</t>

</xml_diff>